<commit_message>
Add level-specific emergency response guidance
</commit_message>
<xml_diff>
--- a/常见化工事故类型与分步应急流程.xlsx
+++ b/常见化工事故类型与分步应急流程.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事故类型速查" sheetId="1" r:id="Re8e72dfbe1654949"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分步应急流程" sheetId="2" r:id="R8384a13634c34bba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="应急处置卡" sheetId="3" r:id="R802a1904076c417e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事故初报与记录" sheetId="4" r:id="R97609d3cdc994e37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明与来源" sheetId="5" r:id="Rdf8cf4a035694ed1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="下拉选项" sheetId="6" r:id="Rf91688b493344758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事故类型速查" sheetId="1" r:id="R09f42f717eea4000"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分步应急流程" sheetId="2" r:id="R9f9651aa95994c25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="应急处置卡" sheetId="3" r:id="R8c986c2dc7de4d43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事故初报与记录" sheetId="4" r:id="Re309c9a448e94075"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明与来源" sheetId="5" r:id="R896911e8c47a4b60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="下拉选项" sheetId="6" r:id="R129c852a2f014ff8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="响应分级措施" sheetId="7" r:id="R14605081a9264056"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +23,7 @@
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="hh:mm"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -51,8 +52,42 @@
       <x:color rgb="FF17365D"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF172033"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF7A4A00"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF172033"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF123A63"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -84,15 +119,83 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF123A63"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF176B9A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF8D7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF0DF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFE6E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="4">
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB8D6E6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB8D6E6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB8D6E6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8D6E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD8E4EA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD8E4EA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD8E4EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E4EA"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -195,6 +298,84 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -359,9 +540,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1435,7 +1616,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6819c0f8c6b044c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R741dfed5a6f24813"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2864,7 +3045,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7eb6565fc6814941"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref0b873f984248e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3894,7 +4075,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13a30f07590b4674"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd225c93861e24720"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4025,6 +4206,38 @@
       </x:c>
       <x:c r="B15" s="28" t="str">
         <x:v>2026-07-13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="36" customHeight="1">
+      <x:c r="A16" s="82" t="str">
+        <x:v>四级颜色说明</x:v>
+      </x:c>
+      <x:c r="B16" s="68" t="str">
+        <x:v>红、橙、黄、蓝用于本系统辅助研判；实际企业响应级别、启动条件、指挥权限和报告程序必须按本单位经评审备案的应急预案及属地规定执行。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="36" customHeight="1">
+      <x:c r="A17" s="82" t="str">
+        <x:v>生产安全事故应急条例</x:v>
+      </x:c>
+      <x:c r="B17" s="68" t="str">
+        <x:v>https://www.mem.gov.cn/fw/flfgbz/fg/201903/t20190301_375884.shtml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="36" customHeight="1">
+      <x:c r="A18" s="82" t="str">
+        <x:v>GB/T 29639—2020说明</x:v>
+      </x:c>
+      <x:c r="B18" s="68" t="str">
+        <x:v>https://www.mem.gov.cn/hd/gzly/lyhf/202308/t20230801_458044.shtml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="36" customHeight="1">
+      <x:c r="A19" s="82" t="str">
+        <x:v>国家突发事件总体应急预案</x:v>
+      </x:c>
+      <x:c r="B19" s="68" t="str">
+        <x:v>https://safety.nanjing.gov.cn/njsaqscjdglj/202503/t20250307_5091091.html</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5038,4 +5251,229 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="17" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="33" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="55" t="str">
+        <x:v>化工事故四级组织响应措施（应用辅助研判）</x:v>
+      </x:c>
+      <x:c r="B1" s="55"/>
+      <x:c r="C1" s="55"/>
+      <x:c r="D1" s="55"/>
+      <x:c r="E1" s="55"/>
+      <x:c r="F1" s="55"/>
+      <x:c r="G1" s="55"/>
+      <x:c r="H1" s="55"/>
+      <x:c r="I1" s="55"/>
+      <x:c r="J1" s="55"/>
+    </x:row>
+    <x:row r="2" ht="44" customHeight="1">
+      <x:c r="A2" s="59" t="str">
+        <x:v>颜色用于本系统辅助研判，不直接等同于法定事故等级或政府响应级别。企业使用时必须按本单位经评审备案的应急预案、属地规定和现场指挥要求完成映射。事故专属处置步骤与本表组织响应措施应同时执行。</x:v>
+      </x:c>
+      <x:c r="B2" s="59"/>
+      <x:c r="C2" s="59"/>
+      <x:c r="D2" s="59"/>
+      <x:c r="E2" s="59"/>
+      <x:c r="F2" s="59"/>
+      <x:c r="G2" s="59"/>
+      <x:c r="H2" s="59"/>
+      <x:c r="I2" s="59"/>
+      <x:c r="J2" s="59"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="51"/>
+      <x:c r="B3" s="51"/>
+      <x:c r="C3" s="51"/>
+      <x:c r="D3" s="51"/>
+      <x:c r="E3" s="51"/>
+      <x:c r="F3" s="51"/>
+      <x:c r="G3" s="51"/>
+      <x:c r="H3" s="51"/>
+      <x:c r="I3" s="51"/>
+      <x:c r="J3" s="51"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="65" t="str">
+        <x:v>颜色等级</x:v>
+      </x:c>
+      <x:c r="B4" s="65" t="str">
+        <x:v>辅助名称</x:v>
+      </x:c>
+      <x:c r="C4" s="65" t="str">
+        <x:v>适用情形</x:v>
+      </x:c>
+      <x:c r="D4" s="65" t="str">
+        <x:v>指挥层级</x:v>
+      </x:c>
+      <x:c r="E4" s="65" t="str">
+        <x:v>报警与报告</x:v>
+      </x:c>
+      <x:c r="F4" s="65" t="str">
+        <x:v>警戒与撤离</x:v>
+      </x:c>
+      <x:c r="G4" s="65" t="str">
+        <x:v>处置力量</x:v>
+      </x:c>
+      <x:c r="H4" s="65" t="str">
+        <x:v>外部联动</x:v>
+      </x:c>
+      <x:c r="I4" s="65" t="str">
+        <x:v>升级条件</x:v>
+      </x:c>
+      <x:c r="J4" s="65" t="str">
+        <x:v>恢复/降级要求</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="96" customHeight="1">
+      <x:c r="A5" s="77" t="str">
+        <x:v>蓝色</x:v>
+      </x:c>
+      <x:c r="B5" s="77" t="str">
+        <x:v>岗位关注响应</x:v>
+      </x:c>
+      <x:c r="C5" s="69" t="str">
+        <x:v>局部异常或少量释放；危险源已停止或可立即隔离；无人员伤害、无扩散，现场监测未超限。</x:v>
+      </x:c>
+      <x:c r="D5" s="69" t="str">
+        <x:v>岗位负责人或班组长组织先期处置，并报告中控。</x:v>
+      </x:c>
+      <x:c r="E5" s="69" t="str">
+        <x:v>立即报告中控/班组长；记录时间、介质、位置和已采取措施。</x:v>
+      </x:c>
+      <x:c r="F5" s="69" t="str">
+        <x:v>隔离作业点，停止无关作业；非必要人员离开危险点并在上风向或安全位置待命。</x:v>
+      </x:c>
+      <x:c r="G5" s="69" t="str">
+        <x:v>仅由受训岗位人员按现场处置卡实施远程停机、切断和监测；不得冒险堵漏。</x:v>
+      </x:c>
+      <x:c r="H5" s="69" t="str">
+        <x:v>企业应急力量备勤；企业预案无特别规定时暂不扩大外部联动。</x:v>
+      </x:c>
+      <x:c r="I5" s="69" t="str">
+        <x:v>不能迅速隔离、报警值上升、影响范围扩大、出现伤情或次生危险。</x:v>
+      </x:c>
+      <x:c r="J5" s="69" t="str">
+        <x:v>危险源隔离、检测合格、泄漏或故障修复，并经班组长/中控确认。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="96" customHeight="1">
+      <x:c r="A6" s="78" t="str">
+        <x:v>黄色</x:v>
+      </x:c>
+      <x:c r="B6" s="78" t="str">
+        <x:v>车间协同响应</x:v>
+      </x:c>
+      <x:c r="C6" s="70" t="str">
+        <x:v>释放持续或影响一个岗位/车间，需要跨岗位协同；尚无严重伤情和厂外影响。</x:v>
+      </x:c>
+      <x:c r="D6" s="70" t="str">
+        <x:v>车间或部门负责人组织处置，企业值班负责人和安全管理人员介入。</x:v>
+      </x:c>
+      <x:c r="E6" s="70" t="str">
+        <x:v>启动车间/现场处置响应；报告企业值班、调度和安全管理部门，持续更新事故信息。</x:v>
+      </x:c>
+      <x:c r="F6" s="70" t="str">
+        <x:v>划定车间或装置警戒区，停止受影响区域作业；疏散非必要人员并清点。</x:v>
+      </x:c>
+      <x:c r="G6" s="70" t="str">
+        <x:v>企业现场应急队、工艺、设备和安全人员协同；消防、医疗力量进入备勤。</x:v>
+      </x:c>
+      <x:c r="H6" s="70" t="str">
+        <x:v>企业应急指挥机构待命；准备119、120、园区及协议救援队联络信息。</x:v>
+      </x:c>
+      <x:c r="I6" s="70" t="str">
+        <x:v>控制失败、监测超限、出现火灾爆炸征兆、人员受伤，或可能扩大至全厂/厂外。</x:v>
+      </x:c>
+      <x:c r="J6" s="70" t="str">
+        <x:v>连续监测合格且无反弹，设备修复完成，由车间负责人会同安全管理人员批准降级。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="96" customHeight="1">
+      <x:c r="A7" s="79" t="str">
+        <x:v>橙色</x:v>
+      </x:c>
+      <x:c r="B7" s="79" t="str">
+        <x:v>企业综合响应</x:v>
+      </x:c>
+      <x:c r="C7" s="71" t="str">
+        <x:v>事故影响装置或厂区，危险源持续释放；需要企业多部门和专业队伍投入，存在次生事故可能。</x:v>
+      </x:c>
+      <x:c r="D7" s="71" t="str">
+        <x:v>企业应急指挥机构启动，由企业负责人或授权现场指挥统一协调。</x:v>
+      </x:c>
+      <x:c r="E7" s="71" t="str">
+        <x:v>启动综合或专项预案；立即报告企业主要负责人，并按规定向有关部门报告事故和响应情况。</x:v>
+      </x:c>
+      <x:c r="F7" s="71" t="str">
+        <x:v>扩大至装置/厂区警戒，组织上风向疏散和人员清点；实施出入口与交通管制。</x:v>
+      </x:c>
+      <x:c r="G7" s="71" t="str">
+        <x:v>企业专业应急队伍、消防、医疗、环境监测和技术专家投入，统一任务和通信。</x:v>
+      </x:c>
+      <x:c r="H7" s="71" t="str">
+        <x:v>根据事故性质请求119、120、协议队伍或园区支援；按规定向属地部门报告并准备周边告知。</x:v>
+      </x:c>
+      <x:c r="I7" s="71" t="str">
+        <x:v>事态失控、多人受伤或重伤、重大火灾爆炸、危险物大量释放，或可能/已经影响厂外。</x:v>
+      </x:c>
+      <x:c r="J7" s="71" t="str">
+        <x:v>危险源受控、救援完成、连续监测合格，经企业应急指挥机构评估后方可降级。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="96" customHeight="1">
+      <x:c r="A8" s="80" t="str">
+        <x:v>红色</x:v>
+      </x:c>
+      <x:c r="B8" s="80" t="str">
+        <x:v>最高级外部联动</x:v>
+      </x:c>
+      <x:c r="C8" s="72" t="str">
+        <x:v>危险源失控；发生重大火灾、爆炸、有毒释放或严重/多人伤亡；已经或可能影响厂外。</x:v>
+      </x:c>
+      <x:c r="D8" s="72" t="str">
+        <x:v>企业启动最高级响应，主要负责人或现场总指挥统一指挥；政府现场指挥部成立后服从统一指挥。</x:v>
+      </x:c>
+      <x:c r="E8" s="72" t="str">
+        <x:v>立即报警并按规定报告；向119、120和属地有关部门提供物质、数量、风险、人员及已采取措施。</x:v>
+      </x:c>
+      <x:c r="F8" s="72" t="str">
+        <x:v>组织全厂及下风向可能受影响区域疏散、清点和交通管制；未经指挥批准任何人不得进入。</x:v>
+      </x:c>
+      <x:c r="G8" s="72" t="str">
+        <x:v>联动消防、医疗、环境监测、专家、园区和政府应急资源；专业队伍在统一指挥下救援。</x:v>
+      </x:c>
+      <x:c r="H8" s="72" t="str">
+        <x:v>全面外部联动；由授权渠道通知可能受影响的周边单位和人员，并持续报告态势。</x:v>
+      </x:c>
+      <x:c r="I8" s="72" t="str">
+        <x:v>本级为最高建议级别；事态变化时持续报告并请求增援，不得擅自降低响应。</x:v>
+      </x:c>
+      <x:c r="J8" s="72" t="str">
+        <x:v>仅在危险源彻底受控、搜救完成、环境与工艺监测合格、结构和设备安全确认后，由统一指挥决定终止或降级。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>